<commit_message>
feat: lengkapi data JK, Tempat Lahir, Tanggal Lahir dari export Dapodik
</commit_message>
<xml_diff>
--- a/import_siswa_sikapdik/Template_Import_Siswa_SIKAPDIK_Kelas1.xlsx
+++ b/import_siswa_sikapdik/Template_Import_Siswa_SIKAPDIK_Kelas1.xlsx
@@ -642,9 +642,21 @@
           <t>Alfarizi Restu Illahi</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Pacitan</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>27/10/2018</t>
+        </is>
+      </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Dusun Sempu, RT 01/RW 07, Desa Jatigunung, Kec. Tulakan, Kab. Pacitan</t>
@@ -670,9 +682,21 @@
           <t>Alif Ramadhan Pratama</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Pekanbaru</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>06/05/2018</t>
+        </is>
+      </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Dusun Nongko, RT 17/RW 09, Desa Gondosari, Kec. Punung, Kab. Pacitan</t>
@@ -698,9 +722,21 @@
           <t>Azizah Khairunisya</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Pacitan</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>08/09/2018</t>
+        </is>
+      </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Dusun Plapar I, RT 03/RW 08, Desa Jatigunung, Kec. Tulakan, Kab. Pacitan</t>
@@ -726,9 +762,21 @@
           <t>Bilqis Naila Fernanda</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Pacitan</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>22/01/2019</t>
+        </is>
+      </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
           <t>RT 01/RW 04, Desa Jatigunung, Kec. Tulakan, Kab. Pacitan</t>
@@ -754,9 +802,21 @@
           <t>Fajar Bagus Setyoaji</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Pacitan</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>23/08/2018</t>
+        </is>
+      </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Dusun Plapar 1, RT 02/RW 08, Desa Jatigunung, Kec. Tulakan, Kab. Pacitan</t>
@@ -782,9 +842,21 @@
           <t>Maher Fadhaililah Ramadhan</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Pacitan</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>09/05/2019</t>
+        </is>
+      </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Dusun Plapar 1, RT 02/RW 08, Desa Jatigunung, Kec. Tulakan, Kab. Pacitan</t>
@@ -810,9 +882,21 @@
           <t>Nadhira Azmi Falisha</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Klaten</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>24/07/2019</t>
+        </is>
+      </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Dusun Plapar 1, RT 01/RW 08, Desa Jatigunung, Kec. Tulakan, Kab. Pacitan</t>
@@ -838,9 +922,21 @@
           <t>Naila Putri Hardiana</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Pacitan</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>23/07/2019</t>
+        </is>
+      </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Dusun Sempu, RT 02/RW 07, Desa Jatigunung, Kec. Tulakan, Kab. Pacitan</t>
@@ -866,9 +962,21 @@
           <t>Nando Arya Saputra</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Pacitan</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>21/09/2018</t>
+        </is>
+      </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Dusun Plapar I, RT 01/RW 08, Desa Jatigunung, Kec. Tulakan, Kab. Pacitan</t>
@@ -894,9 +1002,21 @@
           <t>Syahira Oktaviola Kasih</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr"/>
-      <c r="G14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Pacitan</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>01/10/2018</t>
+        </is>
+      </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Dusun Plapar II, RT 01/RW 08, Desa Jatigunung, Kec. Tulakan, Kab. Pacitan</t>

</xml_diff>